<commit_message>
Stabiler Stand vor UX-Verbesserungen: Vorlagen und Assets aktualisieren.
Master-JSON, neue Garderobenschilder-Assets und Roster-Excel auf den aktuellen Arbeitsstand bringen.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Vorlagen Garderobenschilder/Roster U18 26-27.xlsx
+++ b/Vorlagen Garderobenschilder/Roster U18 26-27.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aaa7f1ebaaab17f6/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noelguyaz/Projekte/Plate-Forge/Vorlagen Garderobenschilder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{D6CF60F8-7D18-804A-88C8-B9359F8454AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{325744D8-11DC-5B4C-9FA9-23B72F0B8907}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2003EF1D-2BDB-D045-BF01-1F4E56A4EA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="19680" windowHeight="17980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>SD</t>
   </si>
@@ -188,9 +188,6 @@
   </si>
   <si>
     <t>Seri</t>
-  </si>
-  <si>
-    <t>Vasile</t>
   </si>
   <si>
     <t>Cserpes</t>
@@ -581,8 +578,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}" name="Tabelle1" displayName="Tabelle1" ref="A1:C33" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" tableBorderDxfId="3">
-  <autoFilter ref="A1:C33" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}" name="Tabelle1" displayName="Tabelle1" ref="A1:C32" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" tableBorderDxfId="3">
+  <autoFilter ref="A1:C32" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{69125100-1D33-9A4E-BB09-D289724DFCD6}" name="Vorname" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{86A36C2A-F7AF-3243-8C89-B3C70121210A}" name="Name" dataDxfId="1"/>
@@ -1634,7 +1631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="18.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.6640625" style="4"/>
@@ -1649,10 +1646,10 @@
         <v>4</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1877,133 +1874,122 @@
     </row>
     <row r="22" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>56</v>
       </c>
       <c r="C22" s="9">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>57</v>
       </c>
       <c r="C23" s="9">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>58</v>
       </c>
       <c r="C24" s="9">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="9">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>60</v>
       </c>
       <c r="C26" s="9">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>61</v>
       </c>
       <c r="C27" s="9">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>62</v>
       </c>
       <c r="C28" s="9">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="9">
-        <v>35</v>
+      <c r="C29" s="10" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>64</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>65</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>66</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C33" s="10" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
U18-Roster aktualisieren und Pokal-Asset zur Bibliothek hinzufügen.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Vorlagen Garderobenschilder/Roster U18 26-27.xlsx
+++ b/Vorlagen Garderobenschilder/Roster U18 26-27.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noelguyaz/Projekte/Plate-Forge/Vorlagen Garderobenschilder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2003EF1D-2BDB-D045-BF01-1F4E56A4EA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2930388-1C98-2743-86DA-CBF24906E6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="19680" windowHeight="17980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="19680" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Roster U18 26-27" sheetId="1" r:id="rId1"/>
+    <sheet name="Roster U21 26-27" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="69">
   <si>
     <t>SD</t>
   </si>
@@ -261,12 +262,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -279,39 +295,7 @@
       <top style="thin">
         <color indexed="10"/>
       </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -322,35 +306,7 @@
       <top style="thin">
         <color indexed="10"/>
       </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -359,14 +315,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -375,32 +328,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <fill>
@@ -410,17 +363,25 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
-          <color indexed="11"/>
+          <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
-          <color indexed="10"/>
+          <color indexed="64"/>
         </top>
         <bottom style="thin">
-          <color indexed="10"/>
+          <color indexed="64"/>
         </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -448,19 +409,25 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
-          <color indexed="10"/>
+          <color indexed="64"/>
         </left>
         <right style="thin">
-          <color indexed="11"/>
+          <color indexed="64"/>
         </right>
         <top style="thin">
-          <color indexed="10"/>
+          <color indexed="64"/>
         </top>
         <bottom style="thin">
-          <color indexed="10"/>
+          <color indexed="64"/>
         </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -472,6 +439,155 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color rgb="FFA5A5A5"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor rgb="FF000000"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border outline="0">
@@ -578,12 +694,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}" name="Tabelle1" displayName="Tabelle1" ref="A1:C32" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" tableBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}" name="Tabelle1" displayName="Tabelle1" ref="A1:C32" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9">
   <autoFilter ref="A1:C32" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{69125100-1D33-9A4E-BB09-D289724DFCD6}" name="Vorname" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{86A36C2A-F7AF-3243-8C89-B3C70121210A}" name="Name" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{707CDD84-EA6D-F04F-9B36-872310499AC8}" name="Nummer" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F90FDF84-6A87-7F4B-9A38-FEC14789254D}" name="Tabelle13" displayName="Tabelle13" ref="A1:C32" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" tableBorderDxfId="6">
+  <autoFilter ref="A1:C32" xr:uid="{56BD9F4F-47DB-3542-A3D9-F89203FA4332}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{9CDADBBC-E125-8943-81DF-B145ECEA65F2}" name="Vorname" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{9DA1F0B0-104F-8A40-B521-95E9DCE83340}" name="Name" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{4B220749-B36E-A04B-9357-2CAD56C46546}" name="Nummer" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1631,367 +1759,562 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="18.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="18.6640625" style="3"/>
+    <col min="2" max="2" width="18.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="15" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" style="3" customWidth="1"/>
+    <col min="5" max="16384" width="18.6640625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="19.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="9">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="9">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="9">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="9">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="9">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="9">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="9">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="9">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A27" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="9">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="9">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A29" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A30" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A32" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A33" s="7"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup orientation="portrait"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000	&amp;P</oddFooter>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00EDC90-AF28-5D42-BB5D-84FCF152CC9B}">
   <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="18.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" style="4"/>
-    <col min="2" max="2" width="18.6640625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="15" style="11" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="18.6640625" style="4"/>
+    <col min="1" max="1" width="18.6640625" style="3"/>
+    <col min="2" max="2" width="18.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="15" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" style="3" customWidth="1"/>
+    <col min="5" max="16384" width="18.6640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="8">
-        <v>1</v>
-      </c>
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="9"/>
     </row>
     <row r="3" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="9">
-        <v>2</v>
-      </c>
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="9"/>
     </row>
     <row r="4" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="9">
-        <v>3</v>
-      </c>
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="9"/>
     </row>
     <row r="5" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="9">
-        <v>4</v>
-      </c>
+      <c r="A5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="9"/>
     </row>
     <row r="6" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="9">
-        <v>5</v>
-      </c>
+      <c r="A6" s="7"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="9"/>
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="9">
-        <v>6</v>
-      </c>
+      <c r="A7" s="7"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="9"/>
     </row>
     <row r="8" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="9">
-        <v>7</v>
-      </c>
+      <c r="A8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="9"/>
     </row>
     <row r="9" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="9">
-        <v>8</v>
-      </c>
+      <c r="A9" s="7"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="9"/>
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="9">
-        <v>9</v>
-      </c>
+      <c r="A10" s="7"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="9"/>
     </row>
     <row r="11" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="9">
-        <v>10</v>
-      </c>
+      <c r="A11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="9"/>
     </row>
     <row r="12" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="9">
-        <v>11</v>
-      </c>
+      <c r="A12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="9"/>
     </row>
     <row r="13" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="9">
-        <v>12</v>
-      </c>
+      <c r="A13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="9"/>
     </row>
     <row r="14" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="9">
-        <v>13</v>
-      </c>
+      <c r="A14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="9"/>
     </row>
     <row r="15" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="9">
-        <v>16</v>
-      </c>
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="9"/>
     </row>
     <row r="16" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="9">
-        <v>17</v>
-      </c>
+      <c r="A16" s="7"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="9"/>
     </row>
     <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="9">
-        <v>20</v>
-      </c>
+      <c r="A17" s="7"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="9"/>
     </row>
     <row r="18" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="9">
-        <v>21</v>
-      </c>
+      <c r="A18" s="7"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="9"/>
     </row>
     <row r="19" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="9">
-        <v>22</v>
-      </c>
+      <c r="A19" s="7"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="9"/>
     </row>
     <row r="20" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="9">
-        <v>23</v>
-      </c>
+      <c r="A20" s="7"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="9"/>
     </row>
     <row r="21" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="9">
-        <v>24</v>
-      </c>
+      <c r="A21" s="7"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="9"/>
     </row>
     <row r="22" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="9">
-        <v>26</v>
-      </c>
+      <c r="A22" s="7"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="9"/>
     </row>
     <row r="23" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C23" s="9">
-        <v>27</v>
-      </c>
+      <c r="A23" s="7"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="9"/>
     </row>
     <row r="24" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C24" s="9">
-        <v>28</v>
-      </c>
+      <c r="A24" s="7"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="9"/>
     </row>
     <row r="25" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" s="9">
-        <v>29</v>
-      </c>
+      <c r="A25" s="7"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="9"/>
     </row>
     <row r="26" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C26" s="9">
-        <v>30</v>
-      </c>
+      <c r="A26" s="7"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="9"/>
     </row>
     <row r="27" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" s="9">
-        <v>31</v>
-      </c>
+      <c r="A27" s="7"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="9"/>
     </row>
     <row r="28" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C28" s="9">
-        <v>35</v>
-      </c>
+      <c r="A28" s="7"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="9"/>
     </row>
     <row r="29" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" s="10" t="s">
-        <v>0</v>
-      </c>
+      <c r="A29" s="7"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="10"/>
     </row>
     <row r="30" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>1</v>
-      </c>
+      <c r="A30" s="7"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="10"/>
     </row>
     <row r="31" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>2</v>
-      </c>
+      <c r="A31" s="7"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="10"/>
     </row>
     <row r="32" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>3</v>
-      </c>
+      <c r="A32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>

</xml_diff>